<commit_message>
manual correction example improvements (+ minor updates)
Manual correction (Excel) example
* improved documentation by adding more detail and adding clear instructions

Code
* made the code less verbose, esp. regarding console output

Documentation
* removed unreachable URLs
* deleted unnecessary PPN sample to decrease repetitions
* restructured content
</commit_message>
<xml_diff>
--- a/spatialnames.xlsx
+++ b/spatialnames.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>NoOfElements</t>
+          <t>ClusterSize</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -461,7 +461,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>AtypicalNoOfElements</t>
+          <t>AtypicalClusterSize</t>
         </is>
       </c>
     </row>

</xml_diff>